<commit_message>
docs: identifica Leonardo no BDD 2 da planilha
</commit_message>
<xml_diff>
--- a/Template_ATDD_Teste_AC1.xlsx
+++ b/Template_ATDD_Teste_AC1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arirosse\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\DevOps_AC1\DevOpsAC1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC85BE0E-B355-4813-BE48-3395D0BAE758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC2A1BF9-B9BB-46CC-83C8-F134B17E0408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pb" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="68">
   <si>
     <t>PRODUCT BACKLOG</t>
   </si>
@@ -472,12 +472,25 @@
   <si>
     <t>ADM (Ariane Rosetti)</t>
   </si>
+  <si>
+    <t>ADM (Leonardo)</t>
+  </si>
+  <si>
+    <t>Aluno concluiu o curso com média 6,9</t>
+  </si>
+  <si>
+    <t>processarEncerramentoDoCurso()</t>
+  </si>
+  <si>
+    <t>temDireitoACursosExtras() = false
+quantidadeCursosExtras = 0</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -567,6 +580,13 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="36"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -746,7 +766,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -845,6 +865,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1062,28 +1085,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S1000"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="1"/>
-    <col min="2" max="2" width="41.54296875" customWidth="1"/>
-    <col min="3" max="3" width="62.26953125" customWidth="1"/>
-    <col min="4" max="4" width="52.453125" customWidth="1"/>
-    <col min="5" max="5" width="46.26953125" customWidth="1"/>
-    <col min="6" max="6" width="13.1796875" customWidth="1"/>
-    <col min="7" max="7" width="53.453125" customWidth="1"/>
-    <col min="8" max="8" width="47.7265625" customWidth="1"/>
-    <col min="9" max="9" width="60.453125" customWidth="1"/>
+    <col min="1" max="1" width="7.21875" customWidth="1"/>
+    <col min="2" max="2" width="41.5546875" customWidth="1"/>
+    <col min="3" max="3" width="62.21875" customWidth="1"/>
+    <col min="4" max="4" width="52.44140625" customWidth="1"/>
+    <col min="5" max="5" width="46.21875" customWidth="1"/>
+    <col min="6" max="6" width="13.21875" customWidth="1"/>
+    <col min="7" max="7" width="53.44140625" customWidth="1"/>
+    <col min="8" max="8" width="47.77734375" customWidth="1"/>
+    <col min="9" max="9" width="60.44140625" customWidth="1"/>
     <col min="10" max="10" width="31" customWidth="1"/>
-    <col min="11" max="11" width="33.1796875" customWidth="1"/>
-    <col min="12" max="12" width="44.1796875" customWidth="1"/>
-    <col min="13" max="13" width="8.453125" customWidth="1"/>
+    <col min="11" max="11" width="33.21875" customWidth="1"/>
+    <col min="12" max="12" width="44.21875" customWidth="1"/>
+    <col min="13" max="13" width="8.44140625" customWidth="1"/>
     <col min="14" max="14" width="169" customWidth="1"/>
-    <col min="15" max="15" width="127.1796875" customWidth="1"/>
-    <col min="16" max="16" width="36.54296875" customWidth="1"/>
+    <col min="15" max="15" width="127.21875" customWidth="1"/>
+    <col min="16" max="16" width="36.5546875" customWidth="1"/>
     <col min="17" max="17" width="39" customWidth="1"/>
-    <col min="18" max="18" width="8.453125" customWidth="1"/>
-    <col min="19" max="19" width="46.26953125" customWidth="1"/>
-    <col min="20" max="26" width="8.453125" customWidth="1"/>
+    <col min="18" max="18" width="8.44140625" customWidth="1"/>
+    <col min="19" max="19" width="46.21875" customWidth="1"/>
+    <col min="20" max="26" width="8.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="55.5" customHeight="1">
@@ -1252,7 +1275,7 @@
     <row r="6" spans="1:19" ht="310.5" customHeight="1">
       <c r="A6" s="9"/>
       <c r="B6" s="21" t="s">
-        <v>18</v>
+        <v>64</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>41</v>
@@ -1279,9 +1302,15 @@
       </c>
       <c r="L6" s="10"/>
       <c r="M6" s="38"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="29"/>
+      <c r="N6" s="43" t="s">
+        <v>65</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="P6" s="29" t="s">
+        <v>67</v>
+      </c>
       <c r="Q6" s="26"/>
       <c r="R6" s="26"/>
       <c r="S6" s="27"/>
@@ -2411,98 +2440,98 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A1000"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="63.26953125" customWidth="1"/>
-    <col min="2" max="26" width="8.453125" customWidth="1"/>
+    <col min="1" max="1" width="63.21875" customWidth="1"/>
+    <col min="2" max="26" width="8.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="58">
+    <row r="1" spans="1:1" ht="57.6">
       <c r="A1" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="14.5">
+    <row r="2" spans="1:1" ht="14.4">
       <c r="A2" s="12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="29">
+    <row r="3" spans="1:1" ht="28.8">
       <c r="A3" s="13" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="14.5">
+    <row r="4" spans="1:1" ht="14.4">
       <c r="A4" s="14"/>
     </row>
-    <row r="5" spans="1:1" ht="14.5">
+    <row r="5" spans="1:1" ht="14.4">
       <c r="A5" s="13" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="14.5">
+    <row r="6" spans="1:1" ht="14.4">
       <c r="A6" s="9"/>
     </row>
-    <row r="7" spans="1:1" ht="14.5">
+    <row r="7" spans="1:1" ht="14.4">
       <c r="A7" s="15" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="14.5">
+    <row r="8" spans="1:1" ht="14.4">
       <c r="A8" s="16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="14.5">
+    <row r="9" spans="1:1" ht="14.4">
       <c r="A9" s="17" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="14.5">
+    <row r="10" spans="1:1" ht="14.4">
       <c r="A10" s="9"/>
     </row>
-    <row r="11" spans="1:1" ht="14.5">
+    <row r="11" spans="1:1" ht="14.4">
       <c r="A11" s="9"/>
     </row>
-    <row r="12" spans="1:1" ht="14.5">
+    <row r="12" spans="1:1" ht="14.4">
       <c r="A12" s="16" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="14.5">
+    <row r="13" spans="1:1" ht="14.4">
       <c r="A13" s="18" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="14.5">
+    <row r="14" spans="1:1" ht="14.4">
       <c r="A14" s="19" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="14.5">
+    <row r="15" spans="1:1" ht="14.4">
       <c r="A15" s="18" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="14.5">
+    <row r="16" spans="1:1" ht="14.4">
       <c r="A16" s="9"/>
     </row>
-    <row r="17" spans="1:1" ht="14.5">
+    <row r="17" spans="1:1" ht="14.4">
       <c r="A17" s="16" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="14.5">
+    <row r="18" spans="1:1" ht="14.4">
       <c r="A18" s="20" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="14.5">
+    <row r="19" spans="1:1" ht="14.4">
       <c r="A19" s="19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="14.5">
+    <row r="20" spans="1:1" ht="14.4">
       <c r="A20" s="18" t="s">
         <v>33</v>
       </c>

</xml_diff>

<commit_message>
reorganiza estrutura de pacotes e pastas da API
</commit_message>
<xml_diff>
--- a/Template_ATDD_Teste_AC1.xlsx
+++ b/Template_ATDD_Teste_AC1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\DevOps_AC1\DevOpsAC1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gabri\OneDrive\Área de Trabalho\facul\DevOpsAC1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC2A1BF9-B9BB-46CC-83C8-F134B17E0408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E49268C2-448D-49B4-9D04-B3BFF7C9296C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pb" sheetId="1" r:id="rId1"/>
@@ -77,9 +77,6 @@
     <t>RESULTS (ASSERTS)</t>
   </si>
   <si>
-    <t>ADM</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -434,9 +431,6 @@
     <t>Dado um aluno que concluiu um curso</t>
   </si>
   <si>
-    <t>E a sua média final foi igual ou superior a 7,0</t>
-  </si>
-  <si>
     <t>Quando o sistema processa o encerramento do curso</t>
   </si>
   <si>
@@ -484,6 +478,12 @@
   <si>
     <t>temDireitoACursosExtras() = false
 quantidadeCursosExtras = 0</t>
+  </si>
+  <si>
+    <t>E a sua média final foi superior a 7,0</t>
+  </si>
+  <si>
+    <t>ADM (Luiz)</t>
   </si>
 </sst>
 </file>
@@ -824,6 +824,9 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -865,9 +868,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1085,104 +1085,104 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S1000"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="7.21875" customWidth="1"/>
-    <col min="2" max="2" width="41.5546875" customWidth="1"/>
-    <col min="3" max="3" width="62.21875" customWidth="1"/>
-    <col min="4" max="4" width="52.44140625" customWidth="1"/>
-    <col min="5" max="5" width="46.21875" customWidth="1"/>
-    <col min="6" max="6" width="13.21875" customWidth="1"/>
-    <col min="7" max="7" width="53.44140625" customWidth="1"/>
-    <col min="8" max="8" width="47.77734375" customWidth="1"/>
-    <col min="9" max="9" width="60.44140625" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" customWidth="1"/>
+    <col min="2" max="2" width="41.5703125" customWidth="1"/>
+    <col min="3" max="3" width="62.28515625" customWidth="1"/>
+    <col min="4" max="4" width="52.42578125" customWidth="1"/>
+    <col min="5" max="5" width="46.28515625" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" customWidth="1"/>
+    <col min="7" max="7" width="53.42578125" customWidth="1"/>
+    <col min="8" max="8" width="47.7109375" customWidth="1"/>
+    <col min="9" max="9" width="60.42578125" customWidth="1"/>
     <col min="10" max="10" width="31" customWidth="1"/>
-    <col min="11" max="11" width="33.21875" customWidth="1"/>
-    <col min="12" max="12" width="44.21875" customWidth="1"/>
-    <col min="13" max="13" width="8.44140625" customWidth="1"/>
+    <col min="11" max="11" width="33.28515625" customWidth="1"/>
+    <col min="12" max="12" width="44.28515625" customWidth="1"/>
+    <col min="13" max="13" width="8.42578125" customWidth="1"/>
     <col min="14" max="14" width="169" customWidth="1"/>
-    <col min="15" max="15" width="127.21875" customWidth="1"/>
-    <col min="16" max="16" width="36.5546875" customWidth="1"/>
+    <col min="15" max="15" width="127.28515625" customWidth="1"/>
+    <col min="16" max="16" width="36.5703125" customWidth="1"/>
     <col min="17" max="17" width="39" customWidth="1"/>
-    <col min="18" max="18" width="8.44140625" customWidth="1"/>
-    <col min="19" max="19" width="46.21875" customWidth="1"/>
-    <col min="20" max="26" width="8.44140625" customWidth="1"/>
+    <col min="18" max="18" width="8.42578125" customWidth="1"/>
+    <col min="19" max="19" width="46.28515625" customWidth="1"/>
+    <col min="20" max="26" width="8.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="55.5" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="27"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="28"/>
       <c r="F1" s="1"/>
-      <c r="G1" s="31" t="s">
+      <c r="G1" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="28"/>
       <c r="M1" s="1"/>
-      <c r="N1" s="32" t="s">
+      <c r="N1" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
-      <c r="R1" s="26"/>
-      <c r="S1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="28"/>
     </row>
     <row r="2" spans="1:19" ht="26.25" customHeight="1">
-      <c r="A2" s="33"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
-      <c r="M2" s="34"/>
-      <c r="N2" s="34"/>
-      <c r="O2" s="34"/>
-      <c r="P2" s="34"/>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="35"/>
+      <c r="A2" s="34"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="36"/>
     </row>
     <row r="3" spans="1:19" ht="36" customHeight="1">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="36" t="s">
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="26"/>
-      <c r="I3" s="26"/>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="27"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="36" t="s">
+      <c r="H3" s="27"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="27"/>
+      <c r="K3" s="27"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="41"/>
+      <c r="N3" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="O3" s="26"/>
-      <c r="P3" s="26"/>
-      <c r="Q3" s="26"/>
-      <c r="R3" s="26"/>
-      <c r="S3" s="27"/>
+      <c r="O3" s="27"/>
+      <c r="P3" s="27"/>
+      <c r="Q3" s="27"/>
+      <c r="R3" s="27"/>
+      <c r="S3" s="28"/>
     </row>
     <row r="4" spans="1:19" ht="66" customHeight="1">
       <c r="A4" s="2" t="s">
@@ -1200,7 +1200,7 @@
       <c r="E4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="38"/>
+      <c r="F4" s="39"/>
       <c r="G4" s="3" t="s">
         <v>11</v>
       </c>
@@ -1219,177 +1219,177 @@
       <c r="L4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="M4" s="38"/>
+      <c r="M4" s="39"/>
       <c r="N4" s="3" t="s">
         <v>15</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="P4" s="42" t="s">
+      <c r="P4" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="Q4" s="26"/>
-      <c r="R4" s="26"/>
-      <c r="S4" s="27"/>
+      <c r="Q4" s="27"/>
+      <c r="R4" s="27"/>
+      <c r="S4" s="28"/>
     </row>
     <row r="5" spans="1:19" ht="409.5" customHeight="1">
       <c r="A5" s="4">
         <v>1</v>
       </c>
       <c r="B5" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="D5" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="E5" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="E5" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="F5" s="38"/>
+      <c r="F5" s="39"/>
       <c r="G5" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="I5" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="J5" s="7"/>
       <c r="K5" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="L5" s="8"/>
-      <c r="M5" s="38"/>
+      <c r="M5" s="39"/>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
-      <c r="P5" s="29"/>
-      <c r="Q5" s="26"/>
-      <c r="R5" s="26"/>
-      <c r="S5" s="27"/>
+      <c r="P5" s="30"/>
+      <c r="Q5" s="27"/>
+      <c r="R5" s="27"/>
+      <c r="S5" s="28"/>
     </row>
     <row r="6" spans="1:19" ht="310.5" customHeight="1">
       <c r="A6" s="9"/>
       <c r="B6" s="21" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C6" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="E6" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="F6" s="38"/>
+      <c r="F6" s="39"/>
       <c r="G6" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="I6" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="J6" s="6"/>
       <c r="K6" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L6" s="10"/>
-      <c r="M6" s="38"/>
-      <c r="N6" s="43" t="s">
+      <c r="M6" s="39"/>
+      <c r="N6" s="25" t="s">
+        <v>63</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P6" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="O6" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="P6" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q6" s="26"/>
-      <c r="R6" s="26"/>
-      <c r="S6" s="27"/>
+      <c r="Q6" s="27"/>
+      <c r="R6" s="27"/>
+      <c r="S6" s="28"/>
     </row>
     <row r="7" spans="1:19" ht="305.25" customHeight="1">
       <c r="A7" s="9"/>
       <c r="B7" s="23" t="s">
-        <v>18</v>
+        <v>67</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D7" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="E7" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E7" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="F7" s="38"/>
+      <c r="F7" s="39"/>
       <c r="G7" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="J7" s="6"/>
       <c r="K7" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L7" s="11"/>
-      <c r="M7" s="38"/>
+      <c r="M7" s="39"/>
       <c r="N7" s="6"/>
       <c r="O7" s="5"/>
-      <c r="P7" s="25"/>
-      <c r="Q7" s="26"/>
-      <c r="R7" s="26"/>
-      <c r="S7" s="27"/>
+      <c r="P7" s="26"/>
+      <c r="Q7" s="27"/>
+      <c r="R7" s="27"/>
+      <c r="S7" s="28"/>
     </row>
     <row r="8" spans="1:19" ht="362.25" customHeight="1">
       <c r="A8" s="9"/>
       <c r="B8" s="23" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="38"/>
+        <v>45</v>
+      </c>
+      <c r="F8" s="39"/>
       <c r="G8" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>60</v>
       </c>
       <c r="J8" s="5"/>
       <c r="K8" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="M8" s="38"/>
+        <v>60</v>
+      </c>
+      <c r="M8" s="39"/>
       <c r="N8" s="6"/>
       <c r="O8" s="5"/>
-      <c r="P8" s="28"/>
-      <c r="Q8" s="26"/>
-      <c r="R8" s="26"/>
-      <c r="S8" s="27"/>
+      <c r="P8" s="29"/>
+      <c r="Q8" s="27"/>
+      <c r="R8" s="27"/>
+      <c r="S8" s="28"/>
     </row>
     <row r="9" spans="1:19" ht="355.5" customHeight="1">
       <c r="A9" s="9"/>
@@ -1397,20 +1397,20 @@
       <c r="C9" s="24"/>
       <c r="D9" s="24"/>
       <c r="E9" s="24"/>
-      <c r="F9" s="38"/>
+      <c r="F9" s="39"/>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
       <c r="L9" s="11"/>
-      <c r="M9" s="38"/>
+      <c r="M9" s="39"/>
       <c r="N9" s="6"/>
       <c r="O9" s="6"/>
-      <c r="P9" s="29"/>
-      <c r="Q9" s="26"/>
-      <c r="R9" s="26"/>
-      <c r="S9" s="27"/>
+      <c r="P9" s="30"/>
+      <c r="Q9" s="27"/>
+      <c r="R9" s="27"/>
+      <c r="S9" s="28"/>
     </row>
     <row r="10" spans="1:19" ht="201" hidden="1" customHeight="1">
       <c r="A10" s="9"/>
@@ -1418,20 +1418,20 @@
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
-      <c r="F10" s="39"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
       <c r="J10" s="9"/>
       <c r="K10" s="9"/>
       <c r="L10" s="9"/>
-      <c r="M10" s="39"/>
+      <c r="M10" s="40"/>
       <c r="N10" s="9"/>
       <c r="O10" s="9"/>
-      <c r="P10" s="41"/>
-      <c r="Q10" s="26"/>
-      <c r="R10" s="26"/>
-      <c r="S10" s="27"/>
+      <c r="P10" s="42"/>
+      <c r="Q10" s="27"/>
+      <c r="R10" s="27"/>
+      <c r="S10" s="28"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -2440,100 +2440,100 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A1000"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="63.21875" customWidth="1"/>
-    <col min="2" max="26" width="8.44140625" customWidth="1"/>
+    <col min="1" max="1" width="63.28515625" customWidth="1"/>
+    <col min="2" max="26" width="8.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="57.6">
+    <row r="1" spans="1:1" ht="60">
       <c r="A1" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="14.4">
-      <c r="A2" s="12" t="s">
+    <row r="3" spans="1:1" ht="30">
+      <c r="A3" s="13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="28.8">
-      <c r="A3" s="13" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="14.4">
+    <row r="4" spans="1:1">
       <c r="A4" s="14"/>
     </row>
-    <row r="5" spans="1:1" ht="14.4">
+    <row r="5" spans="1:1">
       <c r="A5" s="13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="14.4">
+    <row r="6" spans="1:1">
       <c r="A6" s="9"/>
     </row>
-    <row r="7" spans="1:1" ht="14.4">
+    <row r="7" spans="1:1">
       <c r="A7" s="15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" s="16" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="14.4">
-      <c r="A8" s="16" t="s">
+    <row r="9" spans="1:1">
+      <c r="A9" s="17" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="14.4">
-      <c r="A9" s="17" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" ht="14.4">
+    <row r="10" spans="1:1">
       <c r="A10" s="9"/>
     </row>
-    <row r="11" spans="1:1" ht="14.4">
+    <row r="11" spans="1:1">
       <c r="A11" s="9"/>
     </row>
-    <row r="12" spans="1:1" ht="14.4">
+    <row r="12" spans="1:1">
       <c r="A12" s="16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="18" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="14.4">
-      <c r="A13" s="18" t="s">
+    <row r="14" spans="1:1">
+      <c r="A14" s="19" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="14.4">
-      <c r="A14" s="19" t="s">
+    <row r="15" spans="1:1">
+      <c r="A15" s="18" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="14.4">
-      <c r="A15" s="18" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="14.4">
+    <row r="16" spans="1:1">
       <c r="A16" s="9"/>
     </row>
-    <row r="17" spans="1:1" ht="14.4">
+    <row r="17" spans="1:1">
       <c r="A17" s="16" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="14.4">
-      <c r="A18" s="20" t="s">
+    <row r="19" spans="1:1">
+      <c r="A19" s="19" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="14.4">
-      <c r="A19" s="19" t="s">
+    <row r="20" spans="1:1">
+      <c r="A20" s="18" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="14.4">
-      <c r="A20" s="18" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="15.75" customHeight="1">
@@ -2541,17 +2541,17 @@
     </row>
     <row r="22" spans="1:1" ht="15.75" customHeight="1">
       <c r="A22" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="15.75" customHeight="1">
       <c r="A23" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="15.75" customHeight="1">
       <c r="A24" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="15.75" customHeight="1"/>

</xml_diff>